<commit_message>
Handling Device blank values and Device is pointing to dbo.connections.contains
</commit_message>
<xml_diff>
--- a/bos-onboarding/test/DBO_HLI_12_v3.xlsx
+++ b/bos-onboarding/test/DBO_HLI_12_v3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\build2auto\bos-tools\bos-onboarding\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2AF163A-9232-428F-8F92-964EB82ADBA6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2F991C6-BDB8-4F32-8296-A58B1E7926B0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4091" uniqueCount="1035">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4095" uniqueCount="1035">
   <si>
     <t>dbo.section</t>
   </si>
@@ -7626,7 +7626,9 @@
       <c r="W2" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="X2" s="3"/>
+      <c r="X2" s="3" t="s">
+        <v>152</v>
+      </c>
       <c r="Y2" s="3"/>
       <c r="Z2" s="4"/>
       <c r="AA2" s="4"/>
@@ -7689,7 +7691,9 @@
       <c r="W3" t="s">
         <v>622</v>
       </c>
-      <c r="X3" s="3"/>
+      <c r="X3" s="3" t="s">
+        <v>152</v>
+      </c>
       <c r="Y3" s="3"/>
       <c r="Z3" s="4">
         <v>1735869320140</v>
@@ -7754,7 +7758,9 @@
       <c r="W4" t="s">
         <v>623</v>
       </c>
-      <c r="X4" s="3"/>
+      <c r="X4" s="3" t="s">
+        <v>152</v>
+      </c>
       <c r="Y4" s="3"/>
       <c r="Z4" s="4">
         <v>1735869319344</v>
@@ -7819,7 +7825,9 @@
       <c r="W5" t="s">
         <v>624</v>
       </c>
-      <c r="X5" s="3"/>
+      <c r="X5" s="3" t="s">
+        <v>152</v>
+      </c>
       <c r="Y5" s="3"/>
       <c r="Z5" s="4">
         <v>1735869328769</v>

</xml_diff>